<commit_message>
Update battle room and map pipeline
</commit_message>
<xml_diff>
--- a/Tools.Config/GameConfig/Datas/__tables__.xlsx
+++ b/Tools.Config/GameConfig/Datas/__tables__.xlsx
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="3"/>
   <cols>
     <col width="20.3809523809524" customWidth="1" style="2" min="2" max="2"/>
@@ -1198,6 +1198,216 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>battle.TbMap</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>MapConfig</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>map.xlsx</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>mapId</t>
+        </is>
+      </c>
+      <c r="I5" s="0" t="inlineStr">
+        <is>
+          <t>地图配置表：地图资源、人数范围、模式与局内对象约定</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>battle.TbShop</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>ShopConfig</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>shop.xlsx</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>shopId</t>
+        </is>
+      </c>
+      <c r="I6" s="0" t="inlineStr">
+        <is>
+          <t>局内商店表：Tiled shop 层对象通过 shop_id 引用</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>battle.TbShopGoods</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>ShopGoodsConfig</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>shop_goods.xlsx</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>goodsId</t>
+        </is>
+      </c>
+      <c r="I7" s="0" t="inlineStr">
+        <is>
+          <t>局内商店商品表：定义商店售卖物品、价格和解锁条件</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>battle.TbMonster</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>MonsterConfig</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>monster.xlsx</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>monsterId</t>
+        </is>
+      </c>
+      <c r="I8" s="0" t="inlineStr">
+        <is>
+          <t>怪物配置表：Tiled monster 层对象通过 monster_id 引用</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>battle.TbBuilding</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>BuildingConfig</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>building.xlsx</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>buildingId</t>
+        </is>
+      </c>
+      <c r="I9" s="0" t="inlineStr">
+        <is>
+          <t>建筑配置表：建筑类型、预制体、占地、生命值和能力开关</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>battle.TbBuildingLevel</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>BuildingLevelConfig</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>building_level.xlsx</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>levelId</t>
+        </is>
+      </c>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t>建筑卡牌表：局内建造入口、消耗、冷却和展示说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>battle.TbBuildingCard</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>BuildingCardConfig</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>building_card.xlsx</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t>cardId</t>
+        </is>
+      </c>
+      <c r="I11" s="0" t="inlineStr">
+        <is>
+          <t>建筑等级表：升级消耗、生命值、攻击、范围和产出参数</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>

<commit_message>
Sync game systems and widget UI updates
</commit_message>
<xml_diff>
--- a/Tools.Config/GameConfig/Datas/__tables__.xlsx
+++ b/Tools.Config/GameConfig/Datas/__tables__.xlsx
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="3"/>
   <cols>
     <col width="20.3809523809524" customWidth="1" style="2" min="2" max="2"/>
@@ -1231,12 +1231,12 @@
     <row r="6">
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>battle.TbShop</t>
+          <t>battle.TbMonster</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>ShopConfig</t>
+          <t>MonsterConfig</t>
         </is>
       </c>
       <c r="D6" s="0" t="b">
@@ -1244,29 +1244,29 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>shop.xlsx</t>
+          <t>monster.xlsx</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>shopId</t>
+          <t>monsterId</t>
         </is>
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t>局内商店表：Tiled shop 层对象通过 shop_id 引用</t>
+          <t>怪物配置表：Tiled monster 层对象通过 monster_id 引用</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>battle.TbShopGoods</t>
+          <t>battle.TbBuilding</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>ShopGoodsConfig</t>
+          <t>BuildingConfig</t>
         </is>
       </c>
       <c r="D7" s="0" t="b">
@@ -1274,29 +1274,29 @@
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>shop_goods.xlsx</t>
+          <t>building.xlsx</t>
         </is>
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>goodsId</t>
+          <t>buildingId</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>局内商店商品表：定义商店售卖物品、价格和解锁条件</t>
+          <t>建筑配置表：建筑类型、预制体、占地、生命值和能力开关</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>battle.TbMonster</t>
+          <t>battle.TbBuildingLevel</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>MonsterConfig</t>
+          <t>BuildingLevelConfig</t>
         </is>
       </c>
       <c r="D8" s="0" t="b">
@@ -1304,29 +1304,29 @@
       </c>
       <c r="E8" s="0" t="inlineStr">
         <is>
-          <t>monster.xlsx</t>
+          <t>building_level.xlsx</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>monsterId</t>
+          <t>levelId</t>
         </is>
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>怪物配置表：Tiled monster 层对象通过 monster_id 引用</t>
+          <t>建筑卡牌表：局内建造入口、消耗、冷却和展示说明</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>battle.TbBuilding</t>
+          <t>battle.TbBuildingCard</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>BuildingConfig</t>
+          <t>BuildingCardConfig</t>
         </is>
       </c>
       <c r="D9" s="0" t="b">
@@ -1334,29 +1334,29 @@
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t>building.xlsx</t>
+          <t>building_card.xlsx</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>buildingId</t>
+          <t>cardId</t>
         </is>
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t>建筑配置表：建筑类型、预制体、占地、生命值和能力开关</t>
+          <t>建筑等级表：升级消耗、生命值、攻击、范围和产出参数</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>battle.TbBuildingLevel</t>
+          <t>role.TbCharacter</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>BuildingLevelConfig</t>
+          <t>CharacterConfig</t>
         </is>
       </c>
       <c r="D10" s="0" t="b">
@@ -1364,29 +1364,29 @@
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>building_level.xlsx</t>
+          <t>character.xlsx</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>levelId</t>
+          <t>characterId</t>
         </is>
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t>建筑卡牌表：局内建造入口、消耗、冷却和展示说明</t>
+          <t>角色配置表：精灵/巨魔角色、技能、资源和解锁状态</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>battle.TbBuildingCard</t>
+          <t>asset.TbCurrency</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>BuildingCardConfig</t>
+          <t>CurrencyConfig</t>
         </is>
       </c>
       <c r="D11" s="0" t="b">
@@ -1394,17 +1394,227 @@
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t>building_card.xlsx</t>
+          <t>currency.xlsx</t>
         </is>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t>cardId</t>
+          <t>currencyId</t>
         </is>
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t>建筑等级表：升级消耗、生命值、攻击、范围和产出参数</t>
+          <t>局外货币配置表：金币、钻石、活动币等纯数值资产</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>asset.TbItem</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>ItemConfig</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>item.xlsx</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t>itemId</t>
+        </is>
+      </c>
+      <c r="I12" s="0" t="inlineStr">
+        <is>
+          <t>局外道具配置表：票券、体验卡、碎片、增益卡、宝箱和材料</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>open.TbOpenFeature</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>OpenFeatureConfig</t>
+        </is>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>open_feature.xlsx</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>featureId</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>统一开放定义表：活动、功能、限时入口、任务和商店共用</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>shop.TbShop</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ShopConfig</t>
+        </is>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>shop.xlsx</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>shopId</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>局外商店表：常驻、活动和限时商店</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>shop.TbShopGoods</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ShopGoodsConfig</t>
+        </is>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>shop_goods.xlsx</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>goodsId</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>局外商店商品表</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>task.TbTask</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TaskConfig</t>
+        </is>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>task.xlsx</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>taskId</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>局外任务表：每日、周常、成就和活动任务</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>battle.TbBattleShop</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BattleShopConfig</t>
+        </is>
+      </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>battle_shop.xlsx</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>shopId</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>局内商店表：Tiled shop 层对象通过 shop_id 引用</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>battle.TbBattleShopGoods</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BattleShopGoodsConfig</t>
+        </is>
+      </c>
+      <c r="D18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>battle_shop_goods.xlsx</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>goodsId</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>局内商店商品表：定义本局售卖物品、价格和解锁条件</t>
         </is>
       </c>
     </row>

</xml_diff>